<commit_message>
CPHCAPST.CO PP&E + STD
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/CPHCAPST.CO.xlsx
+++ b/data/cox_xlsx/CPHCAPST.CO.xlsx
@@ -7363,8 +7363,14 @@
       <c r="N29" s="16">
         <v>0.0</v>
       </c>
-      <c r="O29" s="16"/>
-      <c r="P29" s="16"/>
+      <c r="O29" s="15">
+        <f t="shared" ref="O29:P29" si="1">O30+O31</f>
+        <v>60.03</v>
+      </c>
+      <c r="P29" s="15">
+        <f t="shared" si="1"/>
+        <v>63.92</v>
+      </c>
       <c r="Q29" s="16"/>
       <c r="R29" s="16"/>
       <c r="S29" s="16"/>

</xml_diff>